<commit_message>
cases: apply 2026-07-13 spec changes + regenerate TestRail import (XML + ID CSV)
Fees & Discounts:
- FD-PERM-009, FD-HIST-006: history-log permission View History Logs -> Work Orders: Create and Edit (log) / Work Order Lines: Create and Edit (line history); precond fixes on FD-HIST-001/005, FD-FLAG-002
- FD-PERM-004: drop removed S13-R11 ref; state Part Sales: C&E + See Financial Data
- NEW FD-TAXN-001/002: taxable jurisdiction note (§5-R15 / S2-R26a / S8-R13)

Simple Flow:
- PO-always-on (Story 2 retired): SF-SET-03, SF-SET-08, SF-QB-02, SF-COMP-06, SF-WOP-03, SF-QB-03, SF-VMIS-01
- Completion gate error-on-click -> disabled+tooltip: SF-COMP-21/22, SF-VAL-11
- VIN removed from completion: SF-VAL-02
- Receive cost/sell-price gate added (S13-R7): SF-RCV-06
- Re-home SF-COMP-01..10 off retired Story 2

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testrail-import/simple-flow-v1-testrail-import.xlsx
+++ b/testrail-import/simple-flow-v1-testrail-import.xlsx
@@ -588,7 +588,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Verify a 'Create Purchase Orders' toggle exists and, when off, hides the Vendor Invoice sub-setting</t>
+          <t>Verify there is no 'Create Purchase Orders' toggle and the Vendor Invoice sub-setting always shows (POs always on)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -614,21 +614,19 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1. Locate a 'Create purchase orders' toggle.
-2. Turn it Off and observe the Vendor Invoice Number setting.
-3. Turn it On and observe the Vendor Invoice Number setting.</t>
+          <t>1. Look for a 'Create purchase orders' toggle in the Work Orders settings.
+2. Locate the Vendor Invoice (Optional/Required) setting.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1. EXPECTED PER SPEC (currently NOT met): a 'Create purchase orders' toggle exists, default On, with helper text.
-2. With Create POs Off, the Vendor Invoice (Optional/Required) sub-setting is hidden and no vendor-invoice capture happens in completion.
-3. With Create POs On, the Vendor Invoice (Optional/Required) sub-setting appears with helper text.</t>
+          <t>1. There is no 'Create purchase orders' toggle — purchase orders are always created for vendor parts (the Create-POs setting and the No-PO/Skip flow were retired).
+2. The Vendor Invoice (Optional/Required) sub-setting always shows with its helper text.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>SV-7696 (S1-R2 (Create purchase orders))</t>
+          <t>SV-7696 (Story 1 / §4 (Create-POs setting retired — POs always on))</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -835,7 +833,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Verify first-use defaults on a brand-new org (auto-approve OFF, create POs ON, vendor invoice REQUIRED)</t>
+          <t>Verify first-use defaults on a brand-new org (auto-approve OFF, vendor invoice REQUIRED; no Create-POs setting)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -862,13 +860,13 @@
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>1. Open /administration/settings → Work Orders tab for the new org.
-2. Read the default state of Auto-approve Lines, Create Purchase Orders, and Vendor Invoice.</t>
+2. Read the default state of Auto-approve Lines and Vendor Invoice.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>1. Auto-approve Lines = OFF (spec default — authoritative).
-2. Create Purchase Orders = ON.
+2. There is no Create Purchase Orders setting — purchase orders are always on.
 3. Vendor Invoice = REQUIRED.</t>
         </is>
       </c>
@@ -1228,7 +1226,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Completion — No-PO / Skip (Story 2)</t>
+          <t>Completion — Simple (Stories 3/4)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1262,7 +1260,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>SV-7697 (S2-R1)</t>
+          <t>SV-7698, SV-7699 (Story 3/4 (streamlined completion — Complete button placement))</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1276,7 +1274,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Completion — No-PO / Skip (Story 2)</t>
+          <t>Completion — Simple (Stories 3/4)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1313,7 +1311,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>SV-7697 (S2-R2 / S2-R3 / S2-R4)</t>
+          <t>SV-7698, SV-7699 (Story 3/4 (streamlined completion — no-parts WO one-confirm))</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1327,7 +1325,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Completion — No-PO / Skip (Story 2)</t>
+          <t>Completion — Simple (Stories 3/4)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1362,7 +1360,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>SV-7697, SV-7710 (S2-R4 / S2-R5 / S15-R3)</t>
+          <t>SV-7698, SV-7699, SV-7710 (Story 3/4 (streamlined completion — Success screen) / S15-R3)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1376,7 +1374,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Completion — No-PO / Skip (Story 2)</t>
+          <t>Completion — Simple (Stories 3/4)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1410,7 +1408,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>SV-7697, SV-7710 (S2-R5 / S15-R3)</t>
+          <t>SV-7698, SV-7699, SV-7710 (Story 3/4 (streamlined completion — Go to Invoice) / S15-R3)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1424,7 +1422,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Completion — No-PO / Skip (Story 2)</t>
+          <t>Completion — Simple (Stories 3/4)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1460,7 +1458,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>SV-7697 (S2-R2 / S2 AC (missing required fields blocked))</t>
+          <t>SV-7698, SV-7699 (Story 3/4 (streamlined completion — missing required fields blocked))</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1469,12 +1467,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Verify with Create POs OFF a work order with vendor parts completes with no PO, no vendor bill and no AP sync</t>
+          <t>Verify a work order with a vendor part creates a PO on completion and routes through the receive step (POs always on)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Completion — No-PO / Skip (Story 2)</t>
+          <t>Completion — Simple (Stories 3/4)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1490,27 +1488,27 @@
       <c r="E22" s="2" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
-2. Create Purchase Orders is set to OFF.
-3. An open work order with an approved vendor-part line exists.</t>
+2. An open work order with an approved vendor-part line exists.
+3. POs are always on — there is no Create-POs setting to turn off.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>1. Complete the work order in one confirm.
-2. Check whether any PO was created.
-3. Check for any vendor bill / AP sync.</t>
+          <t>1. Start completion of the work order.
+2. Observe whether a PO / background order is created for the vendor part and whether receiving is required.
+3. Complete after receiving and check the vendor bill / AP sync.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1. No PO is created.
-2. No vendor bill and no AP sync occur.
-3. No catalog/inventory sync for the vendor/found part; it is received at request time only.</t>
+          <t>1. A PO (background order) is created for the vendor part; Complete Work Order stays disabled until the part is received (S4-R1/R4).
+2. After receiving, completion proceeds and the vendor bill / AP sync occur per the normal pipeline.
+3. There is no skip/no-PO path — the former Create-POs-OFF flow was retired.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>SV-7697 (S2-R6 / S2 AC (Create POs off ⇒ no PO))</t>
+          <t>SV-7698, SV-7699 (Story 3/4 (POs always on — former Create-POs-OFF flow retired))</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1524,7 +1522,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Completion — No-PO / Skip (Story 2)</t>
+          <t>Completion — Simple (Stories 3/4)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1560,7 +1558,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>SV-7697 (S2-R6 / §5 invariant 1)</t>
+          <t>SV-7698, SV-7699 (Story 3/4 (streamlined completion — inventory movement) / §5 invariant 1)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1574,7 +1572,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Completion — No-PO / Skip (Story 2)</t>
+          <t>Completion — Simple (Stories 3/4)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1610,7 +1608,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>SV-7697 (S2-R2 / S2 AC (auto-pick off ⇒ pick in modal))</t>
+          <t>SV-7698, SV-7699 (Story 3/4 (streamlined completion — auto-pick off ⇒ pick in modal))</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1624,7 +1622,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Completion — No-PO / Skip (Story 2)</t>
+          <t>Completion — Simple (Stories 3/4)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1658,7 +1656,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>SV-7697 (S2-R6 / S2 AC (re-open returns to Approved))</t>
+          <t>SV-7698, SV-7699 (Story 3/4 (streamlined completion — re-open returns to Approved))</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1672,7 +1670,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Completion — No-PO / Skip (Story 2)</t>
+          <t>Completion — Simple (Stories 3/4)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1707,7 +1705,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>SV-7697 (S2 AC (individual-line Complete + per-part receive kept))</t>
+          <t>SV-7698, SV-7699 (Story 3/4 (streamlined completion — individual-line Complete + per-part receive))</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -2234,16 +2232,16 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>1. Click Complete Work Order.
-2. Proceed through any tech-story / details gates.
-3. Attempt the final Complete confirm.</t>
+          <t>1. Open the work order with one line in Needs Approval and all other gates satisfied.
+2. Look at the Complete Work Order button and hover it for any tooltip.
+3. Approve the remaining line and re-check the button.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>1. The existing 'you need to approve the line to complete the work order' error appears.
-2. The work order does not complete while a line is unapproved.
-3. There is no new disabled state — the error surfaces on Complete.</t>
+          <t>1. The Complete Work Order button is disabled while any line is unapproved.
+2. A tooltip on the disabled button describes the reason (which line needs approval).
+3. The button enables and completion proceeds once all lines are approved (S4-R8).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2284,15 +2282,15 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm one line is unapproved.
-2. Click Complete Work Order and attempt to complete.
+          <t>1. Confirm one line is unapproved (manually un-approved after being added, Auto-approve ON).
+2. Look at the Complete Work Order button (disabled) and its tooltip.
 3. Re-approve the line and retry.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>1. With the line unapproved, completion is blocked with the approve-line error.
-2. After re-approving all lines, completion proceeds.</t>
+          <t>1. With the line unapproved, the Complete Work Order button is disabled with a tooltip describing the reason.
+2. After re-approving all lines, the button enables and completion proceeds (holds regardless of Auto-approve).</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -3590,7 +3588,7 @@
       <c r="E65" s="2" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
-2. A work order has a vendor part with no vendor assigned and Create POs is on.
+2. A work order has a vendor part with no vendor assigned (purchase orders are always on).
 3. The work order has been completed so POs are generated.</t>
         </is>
       </c>
@@ -5381,20 +5379,22 @@
         <is>
           <t>1. Attempt to receive without a vendor set.
 2. Attempt to receive without a part number.
-3. Attempt to receive without a vendor invoice number.</t>
+3. Attempt to receive with the cost / sell price missing.
+4. Attempt to receive without a vendor invoice number.</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
           <t>1. Receiving is gated until a vendor is set.
-2. Receiving is gated until the missing part number is entered.
-3. Receiving is gated until a vendor invoice number is captured.
-4. On Accept Delivery, cost is editable when $0 or missing (parity with Bulk Receive); the sell-price lock rule is unchanged.</t>
+2. Receiving is gated until the missing part number is entered (S13-R6).
+3. Receiving is gated until a missing cost / sell price is entered (S13-R7).
+4. Receiving is gated until a vendor invoice number is captured.
+5. On Accept Delivery, cost is editable when $0 or missing (parity with Bulk Receive); the sell-price lock rule is unchanged.</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>SV-7707 (S12-R2)</t>
+          <t>SV-7707, SV-7708 (S12-R2 / S13-R6 / S13-R7)</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr"/>
@@ -5951,7 +5951,7 @@
       <c r="E114" s="2" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
-2. A WO with nothing to receive (or POs off) is in the list with the column enabled.</t>
+2. A WO with nothing to receive is in the list with the column enabled.</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
@@ -7414,7 +7414,7 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>Verify completion is blocked when a required VIN is missing (non-review flow)</t>
+          <t>Verify VIN is NOT required at completion in the non-review flow (only mileage and engine hours, when missing)</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -7435,24 +7435,26 @@
       <c r="E145" s="2" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
-2. VIN is required for this org's completion and the work order has no VIN.
-3. Require Review is OFF (VIN is collected at completion in the non-review flow).</t>
+2. Require Review is OFF.
+3. A work order is missing VIN but has mileage and engine hours present.</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>1. Start completion.
-2. Leave VIN empty and try to proceed.</t>
+          <t>1. Start completion and reach the Details step.
+2. Note which vehicle fields are required, then complete with VIN still empty.</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>1. Completion is blocked until the VIN is entered.</t>
+          <t>1. The completion Details step collects only mileage and engine hours (when missing) — VIN is NOT a required completion field (S4-R3).
+2. Completion is NOT blocked by a missing VIN; the work order completes.
+3. VIN is captured later only if Require Review is on, in the Mark Reviewed dialog (Story 16).</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>SV-7698, SV-7710 (S15-R2 / S3-R3)</t>
+          <t>SV-7699 (S4-R3 (VIN removed from completion; captured at Mark Reviewed))</t>
         </is>
       </c>
       <c r="I145" s="2" t="inlineStr"/>
@@ -7868,14 +7870,14 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>1. Click Complete Work Order.
-2. Read the error shown at the final confirm.</t>
+          <t>1. Open a work order with one unapproved line and all other gates satisfied.
+2. Look at the Complete Work Order button and its tooltip.</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>1. The existing 'you need to approve the line to complete the work order' error is shown.
-2. Completion does not proceed until the line is approved.</t>
+          <t>1. The Complete Work Order button is disabled with a tooltip describing which line needs approval.
+2. Completion does not proceed until the line is approved; the button enables once all lines are approved.</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -7937,7 +7939,7 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Verify Create POs OFF produces no PO, vendor bill or AP sync and no catalog/inventory sync</t>
+          <t>Verify there is no Create-POs-OFF bypass — a vendor part always generates a PO and QuickBooks sync on completion</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -7958,26 +7960,27 @@
       <c r="E156" s="2" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
-2. Create Purchase Orders is OFF.
-3. A work order with a vendor/found part exists.</t>
+2. A work order with a vendor/found part exists.
+3. There is no Create Purchase Orders setting to turn off — POs are always on.</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>1. Complete the work order with Create POs OFF.
-2. Check for any PO, vendor bill, AP sync.
-3. Check for any catalog/inventory sync of the vendor/found part.</t>
+          <t>1. Complete the work order that has a vendor/found part (receiving as required).
+2. Check that a PO was created for the vendor part.
+3. Check the vendor bill / AP sync and the catalog/inventory sync.</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>1. No PO, no vendor bill, no AP sync.
-2. No catalog/inventory sync (part is received at request time only).</t>
+          <t>1. A PO is created for the vendor part — no setting suppresses PO creation.
+2. The vendor bill / AP sync occurs per the normal pipeline once received.
+3. Catalog/inventory sync happens per the normal receive pipeline.</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>§5 / §4 (Create POs OFF)</t>
+          <t>§4/§5 (POs always on — no Create-POs-OFF bypass)</t>
         </is>
       </c>
       <c r="I156" s="2" t="inlineStr"/>
@@ -8007,7 +8010,7 @@
       <c r="E157" s="2" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
-2. Create POs is on and a work order has a receivable vendor part.</t>
+2. A work order has a receivable vendor part (purchase orders are always on).</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">

</xml_diff>